<commit_message>
Prezzi non modificabili, prezzo netto finale invisibile nel PDF, optional sempre in italiano (note tradotte)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/data/02_Matrice_Optional_Ferretti.xlsx
+++ b/dist/data/02_Matrice_Optional_Ferretti.xlsx
@@ -6758,7 +6758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6792,6 +6792,11 @@
           <t>Nota</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Nota_IT</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6818,6 +6823,7 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6844,6 +6850,7 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6870,6 +6877,7 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6896,6 +6904,7 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6922,6 +6931,7 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6948,6 +6958,7 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6974,6 +6985,7 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7000,6 +7012,7 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7026,6 +7039,7 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7052,6 +7066,7 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7078,6 +7093,7 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7108,6 +7124,11 @@
           <t>A preliminary assessment of the customer’s tender dimensions and weight is required</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>È necessaria una valutazione preliminare di dimensioni e peso del tender del cliente.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7134,6 +7155,7 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7164,6 +7186,11 @@
           <t>The price refers to the Ferretti Yachts Special Edition version of the Seabob S9. Any alternative configuration will be quoted separately.</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Il prezzo si riferisce alla versione Ferretti Yachts Special Edition del Seabob S9. Qualsiasi configurazione alternativa sarà quotata a parte.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7194,6 +7221,11 @@
           <t>It includes fixing</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Include il fissaggio.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7224,6 +7256,11 @@
           <t>Including fixing</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Fissaggio incluso.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7250,6 +7287,7 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7276,6 +7314,7 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7302,6 +7341,7 @@
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7328,6 +7368,7 @@
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7354,6 +7395,7 @@
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7380,6 +7422,7 @@
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7406,6 +7449,7 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7432,6 +7476,7 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7462,6 +7507,11 @@
           <t>Includes lights for staircase to flybridge and staircases to cockpit, light strips on walkways</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Include le luci della scala per il flybridge e delle scale verso il pozzetto, strisce luminose sui passavanti.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7488,6 +7538,7 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7518,6 +7569,11 @@
           <t>Low profile handrail</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Corrimano a basso profilo.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7544,6 +7600,7 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7570,6 +7627,7 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7596,6 +7654,7 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7622,6 +7681,7 @@
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7648,6 +7708,7 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7674,6 +7735,7 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7700,6 +7762,7 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7726,6 +7789,7 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7752,6 +7816,7 @@
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7782,6 +7847,11 @@
           <t>Colour: White</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Colore: bianco.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7808,6 +7878,7 @@
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7834,6 +7905,7 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7860,6 +7932,7 @@
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7890,6 +7963,11 @@
           <t>Upgrade from 12 to 18 pax</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Upgrade da 12 a 18 persone.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7916,6 +7994,7 @@
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7942,6 +8021,7 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7968,6 +8048,7 @@
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7994,6 +8075,7 @@
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8020,6 +8102,7 @@
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8046,6 +8129,7 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8072,6 +8156,7 @@
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8098,6 +8183,7 @@
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8124,6 +8210,7 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8150,6 +8237,7 @@
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8176,6 +8264,7 @@
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8202,6 +8291,7 @@
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8228,6 +8318,7 @@
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8254,6 +8345,7 @@
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8280,6 +8372,7 @@
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8306,6 +8399,7 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8332,6 +8426,7 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8358,6 +8453,7 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8388,6 +8484,11 @@
           <t>Emergency position indicator radiobeacon (precision type), with hydrostatic, automatic release and activation, I.M.O. approved. Customer required to provide M.M.S.I. for activation. Device cannot operate without connection or activation. Includes onboard GPS sensor, category 1.       After delivery, system activation under Customer’s responsibility.</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Radioboa di localizzazione d'emergenza (tipo di precisione), con rilascio idrostatico automatico e attivazione, approvata I.M.O. Il cliente deve fornire il codice M.M.S.I. per l'attivazione. Il dispositivo non può funzionare senza collegamento o attivazione. Include sensore GPS a bordo, categoria 1. Dopo la consegna l'attivazione del sistema è responsabilità del cliente.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8418,6 +8519,11 @@
           <t>Bow thruster with proportional propellers included</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Include elica di prua con eliche proporzionali.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8444,6 +8550,7 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8470,6 +8577,7 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8496,6 +8604,7 @@
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8526,6 +8635,11 @@
           <t>To be selected only with OPT15208 - Proportional bow thruster upgrade</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Selezionabile solo insieme all'upgrade elica di prua proporzionale (OPT15208).</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8552,6 +8666,7 @@
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8582,6 +8697,11 @@
           <t>The upgrade includes: 4x 16” devo3 monitors on main bridge, 2x 12” evo3 monitors on flybridge</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>L'upgrade include: 4 monitor evo3 da 16” in plancia e 2 monitor evo3 da 12” sul flybridge.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8608,6 +8728,7 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8634,6 +8755,7 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8664,6 +8786,11 @@
           <t>Customer required to provide M.M.S.I. for activation. After delivery, system activation under Customer’s responsibility.</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Il cliente deve fornire il codice M.M.S.I. per l'attivazione. Dopo la consegna l'attivazione del sistema è responsabilità del cliente.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8690,6 +8817,7 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8716,6 +8844,7 @@
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8746,6 +8875,11 @@
           <t>Requires joystick (OPT14747) with bow and stern thrusters, proportional propellers included</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Richiede il joystick (OPT14747) con eliche di prua e di poppa, eliche proporzionali incluse.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8772,6 +8906,7 @@
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8798,6 +8933,7 @@
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8824,6 +8960,7 @@
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8854,6 +8991,11 @@
           <t>Upgrade from std fixed 43”.</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Upgrade dal TV fisso standard da 43”.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8884,6 +9026,11 @@
           <t>Upgrade from std 50”.</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Upgrade dal TV standard da 50”.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8910,6 +9057,7 @@
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8936,6 +9084,7 @@
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8962,6 +9111,7 @@
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8992,6 +9142,11 @@
           <t>Additional in Master</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Aggiuntivo nella cabina armatoriale.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9018,6 +9173,7 @@
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9044,6 +9200,7 @@
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9070,6 +9227,7 @@
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9096,6 +9254,7 @@
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9126,6 +9285,11 @@
           <t>Additional wifi access point and external antenna for full yacht coverage. All electronic devices and cabins will be equipped with wired connections (switch hub POE 24 ports).</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Access point wifi aggiuntivo e antenna esterna per la copertura completa dello yacht. Tutti i dispositivi elettronici e le cabine avranno collegamenti cablati (switch hub POE a 24 porte).</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9156,6 +9320,11 @@
           <t>BOW AREA: No. 2 JL Audio SPEAKERS + FUSION MS400; FLYBRIDGE: No. 4 JL Audio SPEAKERS + 1 AMPLIFIER; COCKPIT: No. 4 JL Audio SPEAKERS + 2 AMPLIFIERS</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>PRUA: 2 altoparlanti JL Audio + FUSION MS400; FLYBRIDGE: 4 altoparlanti JL Audio + 1 amplificatore; POZZETTO: 4 altoparlanti JL Audio + 2 amplificatori.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9182,6 +9351,7 @@
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9212,6 +9382,11 @@
           <t>No. 1 antenna</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>1 antenna.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -9238,6 +9413,7 @@
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9264,6 +9440,7 @@
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9290,6 +9467,7 @@
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9316,6 +9494,7 @@
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9346,6 +9525,11 @@
           <t>Includes Racor filter, smoke separator and 2x22kW generators, upgrade from std 11 kW</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Include filtro Racor, separatore di fumi e 2 generatori da 22 kW, upgrade dallo standard da 11 kW.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9372,6 +9556,7 @@
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9398,6 +9583,7 @@
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9424,6 +9610,7 @@
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -9450,6 +9637,7 @@
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9480,6 +9668,11 @@
           <t>OPT where applicable, as specified in the lighting design plan.</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Dove applicabile, come specificato nel progetto illuminotecnico.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9506,6 +9699,7 @@
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9532,6 +9726,7 @@
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9558,6 +9753,7 @@
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9584,6 +9780,7 @@
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -9610,6 +9807,7 @@
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -9640,6 +9838,11 @@
           <t>Includes lights for staircase to lowerdeck, strip lights under beds</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Include le luci della scala verso il ponte inferiore e le strisce luminose sotto i letti.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9666,6 +9869,7 @@
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9692,6 +9896,7 @@
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9718,6 +9923,7 @@
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9744,6 +9950,7 @@
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9770,6 +9977,7 @@
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9796,6 +10004,7 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9822,6 +10031,7 @@
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9848,6 +10058,7 @@
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9874,6 +10085,7 @@
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9900,6 +10112,7 @@
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9926,6 +10139,7 @@
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -9956,6 +10170,11 @@
           <t>Available for master head only</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Disponibile solo per il bagno armatoriale.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -9982,6 +10201,7 @@
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -10008,6 +10228,7 @@
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -10034,6 +10255,7 @@
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -10060,6 +10282,7 @@
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -10086,6 +10309,7 @@
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -10116,6 +10340,11 @@
           <t>Refrigerator (50 l) on flybridge</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Frigorifero (50 l) sul flybridge.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -10142,6 +10371,7 @@
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -10172,6 +10402,11 @@
           <t>10-bottle capacity wine cellar</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Cantinetta con capacità di 10 bottiglie.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -10202,6 +10437,11 @@
           <t>Includes 1x NG 6 and 1x NG 10.</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Include 1 NG 6 e 1 NG 10.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10228,6 +10468,7 @@
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -10258,6 +10499,11 @@
           <t>Includes: 2 oil filters, 2 gas oil filters, 1 belt, 2 rotors, 2 anodes and 1 carrying case</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Include: 2 filtri olio, 2 filtri gasolio, 1 cinghia, 2 rotori, 2 anodi e 1 valigia.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -10284,6 +10530,7 @@
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -10310,6 +10557,7 @@
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -10336,6 +10584,7 @@
         </is>
       </c>
       <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -10362,6 +10611,7 @@
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -10388,6 +10638,7 @@
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>